<commit_message>
Mise à jour complète du site
</commit_message>
<xml_diff>
--- a/bd_factures_fournisseurs.xlsx
+++ b/bd_factures_fournisseurs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X37"/>
+  <dimension ref="A1:X39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2562,6 +2562,154 @@
       <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr"/>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>B Supplier 1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>C Supplier 1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2002</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Version fonctionnelle sauf bouton créer factures et injection factures fournisseur dans grand livre
</commit_message>
<xml_diff>
--- a/bd_factures_fournisseurs.xlsx
+++ b/bd_factures_fournisseurs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X39"/>
+  <dimension ref="A1:X44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2710,6 +2710,284 @@
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr"/>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Hotel Consulting</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>CCREDIT8</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>as</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>as</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>as</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr"/>
+      <c r="X40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>poposd</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>das</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2025-07-17</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2025-07-18</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2025-07-25</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>sdads</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr"/>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="inlineStr"/>
+      <c r="X41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>baba</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>CCREDIT2</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2025-07-18</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2025-07-18</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2025-07-25</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr"/>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr"/>
+      <c r="X42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Echo Industries</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2000 - Caisse - </t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>tata</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>tata</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>tintin</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr"/>
+      <c r="X43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Hotel Consulting</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>CCREDIT8</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>asf</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>afds</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr"/>
+      <c r="X44" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>